<commit_message>
fix: add missing borders in declaration form header section
Add borders for: S3-S12 right (medium), K4/K6/K8 left, N4/N6/N8 right,
J8 bottom, M11 right, O5/O7 left, S13-S14 right, A14:S14 bottom,
S15-S17 right.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/出口报关单草稿.xlsx
+++ b/output/出口报关单草稿.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,11 @@
     </font>
     <font>
       <name val="宋体"/>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="宋体"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
@@ -50,6 +55,17 @@
     </font>
     <font>
       <name val="宋体"/>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="宋体"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -61,7 +77,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -70,12 +86,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
       <left style="medium"/>
       <top style="medium"/>
     </border>
@@ -102,6 +112,13 @@
       <top style="medium"/>
     </border>
     <border>
+      <top style="medium"/>
+    </border>
+    <border>
+      <right style="medium"/>
+      <top style="medium"/>
+    </border>
+    <border>
       <left style="medium"/>
       <right style="thin"/>
       <bottom style="thin"/>
@@ -137,7 +154,22 @@
       <bottom style="thin"/>
     </border>
     <border>
+      <right style="medium"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
     <border>
       <left style="medium"/>
@@ -185,6 +217,9 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
       <left style="thin"/>
       <right style="thin"/>
     </border>
@@ -193,158 +228,330 @@
       <bottom style="thin"/>
     </border>
     <border>
+      <left style="thin"/>
+      <right style="medium"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
       <left style="medium"/>
+      <bottom style="thin"/>
     </border>
     <border>
       <left style="medium"/>
+    </border>
+    <border>
+      <right style="medium"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
       <right style="medium"/>
       <top style="medium"/>
       <bottom style="medium"/>
     </border>
     <border>
+      <left/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin"/>
-    </border>
-    <border>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
       <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -710,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S34"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.27" customWidth="1" min="1" max="1"/>
@@ -758,7 +965,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>境内发货人</t>
@@ -781,921 +988,928 @@
           <t>(    )</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>出口日期</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>申报日期</t>
         </is>
       </c>
-      <c r="O3" s="7" t="inlineStr">
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>备案号</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="4" t="n"/>
+      <c r="R3" s="4" t="n"/>
+      <c r="S3" s="10" t="n"/>
+    </row>
+    <row r="4" ht="14.25" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>深圳市艾进贸易有限公司</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="12" t="inlineStr"/>
-      <c r="F4" s="11" t="n"/>
-      <c r="G4" s="13" t="inlineStr"/>
-      <c r="H4" s="10" t="n"/>
-      <c r="I4" s="10" t="n"/>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="14" t="inlineStr"/>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="15" t="inlineStr"/>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n"/>
       <c r="K4" s="14" t="inlineStr"/>
-      <c r="L4" s="10" t="n"/>
-      <c r="M4" s="10" t="n"/>
-      <c r="N4" s="10" t="n"/>
-      <c r="O4" s="14" t="inlineStr"/>
-      <c r="P4" s="10" t="n"/>
-      <c r="Q4" s="10" t="n"/>
-      <c r="R4" s="10" t="n"/>
-      <c r="S4" s="10" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="L4" s="12" t="n"/>
+      <c r="M4" s="12" t="n"/>
+      <c r="N4" s="13" t="n"/>
+      <c r="O4" s="16" t="inlineStr"/>
+      <c r="P4" s="12" t="n"/>
+      <c r="Q4" s="12" t="n"/>
+      <c r="R4" s="12" t="n"/>
+      <c r="S4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="12" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>境外收货人</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>运输方式</t>
         </is>
       </c>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>(    )</t>
         </is>
       </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="G5" s="23" t="inlineStr">
         <is>
           <t>运输工具名称及航次号</t>
         </is>
       </c>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="21" t="n"/>
-      <c r="K5" s="18" t="inlineStr">
+      <c r="H5" s="19" t="n"/>
+      <c r="I5" s="19" t="n"/>
+      <c r="J5" s="24" t="n"/>
+      <c r="K5" s="21" t="inlineStr">
         <is>
           <t>提运单号</t>
         </is>
       </c>
+      <c r="O5" s="21" t="inlineStr"/>
+      <c r="P5" s="19" t="n"/>
+      <c r="Q5" s="25" t="inlineStr"/>
+      <c r="R5" s="19" t="n"/>
+      <c r="S5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>ZEATALINE INTERNATIONAL TRADING</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="23" t="inlineStr">
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>水路运输</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
-      <c r="J6" s="10" t="n"/>
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="15" t="inlineStr"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
       <c r="K6" s="14" t="inlineStr"/>
-      <c r="L6" s="10" t="n"/>
-      <c r="M6" s="10" t="n"/>
-      <c r="N6" s="10" t="n"/>
-      <c r="O6" s="14" t="inlineStr"/>
-      <c r="P6" s="10" t="n"/>
-      <c r="Q6" s="10" t="n"/>
-      <c r="R6" s="10" t="n"/>
-      <c r="S6" s="10" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="L6" s="12" t="n"/>
+      <c r="M6" s="12" t="n"/>
+      <c r="N6" s="13" t="n"/>
+      <c r="O6" s="16" t="inlineStr"/>
+      <c r="P6" s="12" t="n"/>
+      <c r="Q6" s="12" t="n"/>
+      <c r="R6" s="12" t="n"/>
+      <c r="S6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="12" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>生产销售单位</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="B7" s="19" t="n"/>
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>监管方式</t>
         </is>
       </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>(    )</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>征免性质</t>
         </is>
       </c>
-      <c r="H7" s="24" t="inlineStr">
+      <c r="H7" s="30" t="inlineStr">
         <is>
           <t>(    )</t>
         </is>
       </c>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="21" t="n"/>
-      <c r="K7" s="18" t="inlineStr">
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="24" t="n"/>
+      <c r="K7" s="21" t="inlineStr">
         <is>
           <t>许可证号</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="O7" s="21" t="inlineStr"/>
+      <c r="P7" s="25" t="inlineStr"/>
+      <c r="Q7" s="19" t="n"/>
+      <c r="R7" s="19" t="n"/>
+      <c r="S7" s="26" t="n"/>
+    </row>
+    <row r="8" ht="14.25" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>深圳市艾进贸易有限公司</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="25" t="inlineStr">
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>一般贸易</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="26" t="inlineStr">
+      <c r="F8" s="13" t="n"/>
+      <c r="G8" s="32" t="inlineStr">
         <is>
           <t>一般征税</t>
         </is>
       </c>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="33" t="inlineStr"/>
       <c r="K8" s="14" t="inlineStr"/>
-      <c r="L8" s="10" t="n"/>
-      <c r="M8" s="10" t="n"/>
-      <c r="N8" s="10" t="n"/>
-      <c r="O8" s="14" t="inlineStr"/>
-      <c r="P8" s="10" t="n"/>
-      <c r="Q8" s="10" t="n"/>
-      <c r="R8" s="10" t="n"/>
-      <c r="S8" s="10" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="13" t="n"/>
+      <c r="O8" s="16" t="inlineStr"/>
+      <c r="P8" s="12" t="n"/>
+      <c r="Q8" s="12" t="n"/>
+      <c r="R8" s="12" t="n"/>
+      <c r="S8" s="17" t="n"/>
+    </row>
+    <row r="9" ht="12" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>合同协议号</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n"/>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="n"/>
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>贸易国(地区)</t>
         </is>
       </c>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>(  USA  )</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>运抵国（地区）</t>
         </is>
       </c>
-      <c r="H9" s="27" t="inlineStr">
+      <c r="H9" s="34" t="inlineStr">
         <is>
           <t>(  USA  )</t>
         </is>
       </c>
-      <c r="K9" s="18" t="inlineStr">
+      <c r="K9" s="21" t="inlineStr">
         <is>
           <t>指运港</t>
         </is>
       </c>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>(    )</t>
         </is>
       </c>
-      <c r="M9" s="16" t="n"/>
-      <c r="N9" s="21" t="n"/>
-      <c r="O9" s="18" t="inlineStr">
+      <c r="M9" s="19" t="n"/>
+      <c r="N9" s="24" t="n"/>
+      <c r="O9" s="35" t="inlineStr">
         <is>
           <t>离境口岸</t>
         </is>
       </c>
-      <c r="P9" s="28" t="inlineStr">
+      <c r="P9" s="36" t="inlineStr">
         <is>
           <t>(    )</t>
         </is>
       </c>
-      <c r="Q9" s="16" t="n"/>
-      <c r="R9" s="16" t="n"/>
-      <c r="S9" s="29" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="26" t="n"/>
+    </row>
+    <row r="10" ht="14.25" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>PO2603230466</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="25" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="37" t="inlineStr">
         <is>
           <t>美国</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="30" t="inlineStr">
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="38" t="inlineStr">
         <is>
           <t>美国</t>
         </is>
       </c>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="23" t="inlineStr">
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="28" t="inlineStr">
         <is>
           <t>美国</t>
         </is>
       </c>
-      <c r="L10" s="10" t="n"/>
-      <c r="M10" s="10" t="n"/>
-      <c r="N10" s="11" t="n"/>
-      <c r="O10" s="14" t="inlineStr"/>
-      <c r="P10" s="10" t="n"/>
-      <c r="Q10" s="10" t="n"/>
-      <c r="R10" s="10" t="n"/>
-      <c r="S10" s="10" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="L10" s="12" t="n"/>
+      <c r="M10" s="12" t="n"/>
+      <c r="N10" s="13" t="n"/>
+      <c r="O10" s="16" t="inlineStr"/>
+      <c r="P10" s="12" t="n"/>
+      <c r="Q10" s="12" t="n"/>
+      <c r="R10" s="12" t="n"/>
+      <c r="S10" s="17" t="n"/>
+    </row>
+    <row r="11" ht="12" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>包装种类</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n"/>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>( 22/06   )</t>
         </is>
       </c>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="39" t="inlineStr">
         <is>
           <t>件数</t>
         </is>
       </c>
-      <c r="F11" s="32" t="inlineStr">
+      <c r="F11" s="40" t="inlineStr">
         <is>
           <t>毛重（千克）</t>
         </is>
       </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>净重（千克）</t>
         </is>
       </c>
-      <c r="H11" s="21" t="n"/>
-      <c r="I11" s="33" t="inlineStr">
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="41" t="inlineStr">
         <is>
           <t>成交方式</t>
         </is>
       </c>
-      <c r="K11" s="18" t="inlineStr">
+      <c r="J11" s="42" t="inlineStr">
+        <is>
+          <t>(  )</t>
+        </is>
+      </c>
+      <c r="K11" s="21" t="inlineStr">
         <is>
           <t>运费</t>
         </is>
       </c>
-      <c r="N11" s="34" t="inlineStr">
+      <c r="L11" s="43" t="inlineStr"/>
+      <c r="M11" s="24" t="n"/>
+      <c r="N11" s="42" t="inlineStr">
         <is>
           <t>保费</t>
         </is>
       </c>
-      <c r="Q11" s="18" t="inlineStr">
+      <c r="Q11" s="21" t="inlineStr">
         <is>
           <t>杂费</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="R11" s="25" t="inlineStr"/>
+      <c r="S11" s="26" t="n"/>
+    </row>
+    <row r="12" ht="14.25" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>纸制或纤维板制盒/箱/包/袋</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="25" t="n">
-        <v>43</v>
-      </c>
-      <c r="F12" s="25" t="n">
-        <v>944.8</v>
-      </c>
-      <c r="G12" s="25" t="n">
-        <v>761.4</v>
-      </c>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="26" t="inlineStr">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="31" t="n">
+        <v>900</v>
+      </c>
+      <c r="F12" s="31" t="n">
+        <v>7260</v>
+      </c>
+      <c r="G12" s="31" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="32" t="inlineStr">
         <is>
           <t>CNF</t>
         </is>
       </c>
-      <c r="J12" s="10" t="n"/>
-      <c r="K12" s="35" t="inlineStr">
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="44" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="L12" s="36" t="n">
-        <v>2037.82</v>
-      </c>
-      <c r="M12" s="11" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="37" t="inlineStr">
+      <c r="L12" s="45" t="n">
+        <v>16611.93</v>
+      </c>
+      <c r="M12" s="13" t="n"/>
+      <c r="N12" s="46" t="n"/>
+      <c r="O12" s="12" t="n"/>
+      <c r="P12" s="13" t="n"/>
+      <c r="Q12" s="47" t="n"/>
+      <c r="R12" s="12" t="n"/>
+      <c r="S12" s="17" t="n"/>
+    </row>
+    <row r="13" ht="12" customHeight="1">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>随附单证及编号</t>
         </is>
       </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="19" t="n"/>
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="19" t="n"/>
+      <c r="L13" s="19" t="n"/>
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="19" t="n"/>
+      <c r="O13" s="19" t="n"/>
+      <c r="P13" s="19" t="n"/>
+      <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="12.75" customHeight="1">
+      <c r="A14" s="49" t="inlineStr"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="16" t="inlineStr"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12" t="n"/>
+      <c r="M14" s="12" t="n"/>
+      <c r="N14" s="12" t="n"/>
+      <c r="O14" s="12" t="n"/>
+      <c r="P14" s="12" t="n"/>
+      <c r="Q14" s="12" t="n"/>
+      <c r="R14" s="12" t="n"/>
+      <c r="S14" s="17" t="n"/>
+    </row>
+    <row r="15" ht="12" customHeight="1">
+      <c r="A15" s="50" t="inlineStr">
         <is>
           <t>标记唛码及备注：</t>
         </is>
       </c>
+      <c r="C15" s="51" t="inlineStr"/>
+      <c r="S15" s="52" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" s="50" t="inlineStr">
         <is>
           <t>备注：</t>
         </is>
       </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="39" t="n"/>
-      <c r="B18" s="39" t="n"/>
-      <c r="C18" s="39" t="n"/>
-      <c r="D18" s="39" t="n"/>
-      <c r="E18" s="39" t="n"/>
-      <c r="F18" s="39" t="n"/>
-      <c r="G18" s="39" t="n"/>
-      <c r="H18" s="39" t="n"/>
-      <c r="I18" s="39" t="n"/>
-      <c r="J18" s="39" t="n"/>
-      <c r="K18" s="39" t="n"/>
-      <c r="L18" s="39" t="n"/>
-      <c r="M18" s="39" t="n"/>
-      <c r="N18" s="39" t="n"/>
-      <c r="O18" s="39" t="n"/>
-      <c r="P18" s="39" t="n"/>
-      <c r="Q18" s="39" t="n"/>
-      <c r="R18" s="39" t="n"/>
-      <c r="S18" s="39" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="40" t="inlineStr">
+      <c r="B16" s="51" t="inlineStr"/>
+      <c r="S16" s="52" t="n"/>
+    </row>
+    <row r="17" ht="14.25" customHeight="1">
+      <c r="A17" s="53" t="inlineStr"/>
+      <c r="O17" s="51" t="inlineStr"/>
+      <c r="S17" s="52" t="n"/>
+    </row>
+    <row r="18" ht="14.25" customHeight="1">
+      <c r="A18" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B18" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C18" s="56" t="n"/>
+      <c r="D18" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E18" s="56" t="n"/>
+      <c r="F18" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="G18" s="59" t="n"/>
+      <c r="H18" s="56" t="n"/>
+      <c r="I18" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J18" s="59" t="n"/>
+      <c r="K18" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L18" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="M18" s="59" t="n"/>
+      <c r="N18" s="59" t="n"/>
+      <c r="O18" s="59" t="n"/>
+      <c r="P18" s="59" t="n"/>
+      <c r="Q18" s="59" t="n"/>
+      <c r="R18" s="59" t="n"/>
+      <c r="S18" s="62" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="63" t="inlineStr">
         <is>
           <t>项号</t>
         </is>
       </c>
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="64" t="inlineStr">
         <is>
           <t>商品编号</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="41" t="inlineStr">
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="65" t="inlineStr">
         <is>
           <t>商品名称及规格型号</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="41" t="inlineStr">
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="65" t="inlineStr">
         <is>
           <t>数量及单位</t>
         </is>
       </c>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="41" t="inlineStr">
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="64" t="inlineStr">
         <is>
           <t>单价/总价/币制</t>
         </is>
       </c>
-      <c r="J19" s="10" t="n"/>
-      <c r="K19" s="41" t="inlineStr">
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="65" t="inlineStr">
         <is>
           <t>原产国（地区）</t>
         </is>
       </c>
-      <c r="L19" s="10" t="n"/>
-      <c r="M19" s="41" t="inlineStr">
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="65" t="inlineStr">
         <is>
           <t>最终目的国（地区）</t>
         </is>
       </c>
-      <c r="N19" s="10" t="n"/>
-      <c r="O19" s="10" t="n"/>
-      <c r="P19" s="41" t="inlineStr">
+      <c r="N19" s="12" t="n"/>
+      <c r="O19" s="12" t="n"/>
+      <c r="P19" s="64" t="inlineStr">
         <is>
           <t>境内货源地</t>
         </is>
       </c>
-      <c r="Q19" s="10" t="n"/>
-      <c r="R19" s="10" t="n"/>
-      <c r="S19" s="42" t="inlineStr">
+      <c r="Q19" s="12" t="n"/>
+      <c r="R19" s="12" t="n"/>
+      <c r="S19" s="66" t="inlineStr">
         <is>
           <t>征免</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="43" t="n">
+    <row r="20" ht="14.25" customHeight="1">
+      <c r="A20" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="44" t="n">
-        <v>3918909001</v>
-      </c>
-      <c r="D20" s="44" t="inlineStr">
-        <is>
-          <t>仿真草坪</t>
-        </is>
-      </c>
-      <c r="G20" s="45" t="n">
-        <v>125</v>
-      </c>
-      <c r="H20" s="45" t="inlineStr">
+      <c r="B20" s="68" t="inlineStr">
+        <is>
+          <t>3918909000</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="68" t="inlineStr">
+        <is>
+          <t>人造草坪拼接地板</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="69" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H20" s="69" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="I20" s="46" t="n">
-        <v>4.577313</v>
-      </c>
-      <c r="K20" s="47" t="inlineStr">
+      <c r="I20" s="70" t="n">
+        <v>6.034697</v>
+      </c>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="71" t="inlineStr">
         <is>
           <t>中国</t>
         </is>
       </c>
-      <c r="M20" s="48" t="inlineStr">
+      <c r="L20" s="19" t="n"/>
+      <c r="M20" s="72" t="inlineStr">
         <is>
           <t>美国</t>
         </is>
       </c>
-      <c r="P20" s="48" t="inlineStr">
+      <c r="N20" s="19" t="n"/>
+      <c r="O20" s="19" t="n"/>
+      <c r="P20" s="72" t="inlineStr">
         <is>
           <t>义乌(33189)</t>
         </is>
       </c>
-      <c r="S20" s="49" t="inlineStr">
+      <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="73" t="inlineStr">
         <is>
           <t>照章征税</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="D21" s="50" t="inlineStr">
-        <is>
-          <t>0|0|塑料|塑料草坪|无品牌|无型号</t>
-        </is>
-      </c>
-      <c r="G21" s="45" t="n">
-        <v>75</v>
-      </c>
-      <c r="H21" s="45" t="inlineStr">
+      <c r="A21" s="74" t="n"/>
+      <c r="B21" s="75" t="n"/>
+      <c r="D21" s="76" t="inlineStr">
+        <is>
+          <t>0|0|塑料|人造草坪拼接地板|无品牌|无型号</t>
+        </is>
+      </c>
+      <c r="G21" s="77" t="n">
+        <v>2550</v>
+      </c>
+      <c r="H21" s="77" t="inlineStr">
         <is>
           <t>千克</t>
         </is>
       </c>
-      <c r="I21" s="46" t="n">
-        <v>572.16</v>
-      </c>
-      <c r="K21" s="47" t="inlineStr">
+      <c r="I21" s="78" t="n">
+        <v>21724.91</v>
+      </c>
+      <c r="K21" s="79" t="inlineStr">
         <is>
           <t>（CHN）</t>
         </is>
       </c>
-      <c r="M21" s="47" t="inlineStr">
+      <c r="M21" s="79" t="inlineStr">
         <is>
           <t>（USA）</t>
         </is>
       </c>
+      <c r="P21" s="75" t="n"/>
+      <c r="S21" s="80" t="n"/>
     </row>
     <row r="22">
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="51" t="n">
-        <v>125</v>
-      </c>
-      <c r="H22" s="51" t="inlineStr">
+      <c r="A22" s="81" t="n"/>
+      <c r="B22" s="82" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="83" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H22" s="83" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="I22" s="52" t="inlineStr">
+      <c r="I22" s="84" t="inlineStr">
         <is>
           <t>美元</t>
         </is>
       </c>
-      <c r="J22" s="10" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="43" t="n">
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="82" t="n"/>
+      <c r="L22" s="12" t="n"/>
+      <c r="M22" s="82" t="n"/>
+      <c r="N22" s="12" t="n"/>
+      <c r="O22" s="12" t="n"/>
+      <c r="P22" s="82" t="n"/>
+      <c r="Q22" s="12" t="n"/>
+      <c r="R22" s="12" t="n"/>
+      <c r="S22" s="85" t="n"/>
+    </row>
+    <row r="23" ht="14.25" customHeight="1">
+      <c r="A23" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="B23" s="44" t="n">
-        <v>3918909001</v>
-      </c>
-      <c r="D23" s="44" t="inlineStr">
-        <is>
-          <t>仿真草坪</t>
-        </is>
-      </c>
-      <c r="G23" s="45" t="n">
-        <v>192</v>
-      </c>
-      <c r="H23" s="45" t="inlineStr">
+      <c r="B23" s="68" t="inlineStr">
+        <is>
+          <t>3926909090</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="68" t="inlineStr">
+        <is>
+          <t>塑料草坪围栏</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="69" t="n">
+        <v>2400</v>
+      </c>
+      <c r="H23" s="69" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="I23" s="46" t="n">
-        <v>9.308795999999999</v>
-      </c>
-      <c r="K23" s="47" t="inlineStr">
+      <c r="I23" s="70" t="n">
+        <v>5.643881</v>
+      </c>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="71" t="inlineStr">
         <is>
           <t>中国</t>
         </is>
       </c>
-      <c r="M23" s="48" t="inlineStr">
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="72" t="inlineStr">
         <is>
           <t>美国</t>
         </is>
       </c>
-      <c r="P23" s="48" t="inlineStr">
+      <c r="N23" s="19" t="n"/>
+      <c r="O23" s="19" t="n"/>
+      <c r="P23" s="72" t="inlineStr">
         <is>
           <t>义乌(33189)</t>
         </is>
       </c>
-      <c r="S23" s="49" t="inlineStr">
+      <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="73" t="inlineStr">
         <is>
           <t>照章征税</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="D24" s="50" t="inlineStr">
-        <is>
-          <t>0|0|塑料|塑料草坪|无品牌|无型号</t>
-        </is>
-      </c>
-      <c r="G24" s="45" t="n">
-        <v>230.4</v>
-      </c>
-      <c r="H24" s="45" t="inlineStr">
+      <c r="A24" s="74" t="n"/>
+      <c r="B24" s="75" t="n"/>
+      <c r="D24" s="76" t="inlineStr">
+        <is>
+          <t>0|0|塑料|塑料草坪围栏|无品牌|无型号</t>
+        </is>
+      </c>
+      <c r="G24" s="77" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H24" s="77" t="inlineStr">
         <is>
           <t>千克</t>
         </is>
       </c>
-      <c r="I24" s="46" t="n">
-        <v>1787.29</v>
-      </c>
-      <c r="K24" s="47" t="inlineStr">
+      <c r="I24" s="78" t="n">
+        <v>13545.31</v>
+      </c>
+      <c r="K24" s="79" t="inlineStr">
         <is>
           <t>（CHN）</t>
         </is>
       </c>
-      <c r="M24" s="47" t="inlineStr">
+      <c r="M24" s="79" t="inlineStr">
         <is>
           <t>（USA）</t>
         </is>
       </c>
+      <c r="P24" s="75" t="n"/>
+      <c r="S24" s="80" t="n"/>
     </row>
     <row r="25">
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="51" t="n">
-        <v>192</v>
-      </c>
-      <c r="H25" s="51" t="inlineStr">
+      <c r="A25" s="81" t="n"/>
+      <c r="B25" s="82" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="83" t="n">
+        <v>2400</v>
+      </c>
+      <c r="H25" s="83" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="I25" s="52" t="inlineStr">
+      <c r="I25" s="84" t="inlineStr">
         <is>
           <t>美元</t>
         </is>
       </c>
-      <c r="J25" s="10" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="43" t="n">
+      <c r="J25" s="12" t="n"/>
+      <c r="K25" s="82" t="n"/>
+      <c r="L25" s="12" t="n"/>
+      <c r="M25" s="82" t="n"/>
+      <c r="N25" s="12" t="n"/>
+      <c r="O25" s="12" t="n"/>
+      <c r="P25" s="82" t="n"/>
+      <c r="Q25" s="12" t="n"/>
+      <c r="R25" s="12" t="n"/>
+      <c r="S25" s="85" t="n"/>
+    </row>
+    <row r="26" ht="14.25" customHeight="1">
+      <c r="A26" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="B26" s="44" t="n">
-        <v>3918909001</v>
-      </c>
-      <c r="D26" s="44" t="inlineStr">
-        <is>
-          <t>仿真草坪</t>
-        </is>
-      </c>
-      <c r="G26" s="45" t="n">
-        <v>66</v>
-      </c>
-      <c r="H26" s="45" t="inlineStr">
+      <c r="B26" s="68" t="inlineStr">
+        <is>
+          <t>6702100000</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="68" t="inlineStr">
+        <is>
+          <t>仿真植物墙装饰</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="69" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H26" s="69" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="I26" s="46" t="n">
-        <v>20.409274</v>
-      </c>
-      <c r="K26" s="47" t="inlineStr">
+      <c r="I26" s="70" t="n">
+        <v>7.984399</v>
+      </c>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="71" t="inlineStr">
         <is>
           <t>中国</t>
         </is>
       </c>
-      <c r="M26" s="48" t="inlineStr">
+      <c r="L26" s="19" t="n"/>
+      <c r="M26" s="72" t="inlineStr">
         <is>
           <t>美国</t>
         </is>
       </c>
-      <c r="P26" s="48" t="inlineStr">
+      <c r="N26" s="19" t="n"/>
+      <c r="O26" s="19" t="n"/>
+      <c r="P26" s="72" t="inlineStr">
         <is>
           <t>义乌(33189)</t>
         </is>
       </c>
-      <c r="S26" s="49" t="inlineStr">
+      <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="73" t="inlineStr">
         <is>
           <t>照章征税</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="D27" s="50" t="inlineStr">
-        <is>
-          <t>0|0|塑料|塑料草坪|无品牌|无型号</t>
-        </is>
-      </c>
-      <c r="G27" s="45" t="n">
-        <v>198</v>
-      </c>
-      <c r="H27" s="45" t="inlineStr">
+      <c r="A27" s="74" t="n"/>
+      <c r="B27" s="75" t="n"/>
+      <c r="D27" s="76" t="inlineStr">
+        <is>
+          <t>0|0|塑料|仿真植物墙|无品牌|无型号</t>
+        </is>
+      </c>
+      <c r="G27" s="77" t="n">
+        <v>1950</v>
+      </c>
+      <c r="H27" s="77" t="inlineStr">
         <is>
           <t>千克</t>
         </is>
       </c>
-      <c r="I27" s="46" t="n">
-        <v>1347.01</v>
-      </c>
-      <c r="K27" s="47" t="inlineStr">
+      <c r="I27" s="78" t="n">
+        <v>14371.92</v>
+      </c>
+      <c r="K27" s="79" t="inlineStr">
         <is>
           <t>（CHN）</t>
         </is>
       </c>
-      <c r="M27" s="47" t="inlineStr">
+      <c r="M27" s="79" t="inlineStr">
         <is>
           <t>（USA）</t>
         </is>
       </c>
+      <c r="P27" s="75" t="n"/>
+      <c r="S27" s="80" t="n"/>
     </row>
     <row r="28">
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="51" t="n">
-        <v>66</v>
-      </c>
-      <c r="H28" s="51" t="inlineStr">
+      <c r="A28" s="81" t="n"/>
+      <c r="B28" s="82" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="83" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H28" s="83" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="I28" s="52" t="inlineStr">
+      <c r="I28" s="84" t="inlineStr">
         <is>
           <t>美元</t>
         </is>
       </c>
-      <c r="J28" s="10" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="43" t="n">
-        <v>4</v>
-      </c>
-      <c r="B29" s="44" t="n">
-        <v>3918909001</v>
-      </c>
-      <c r="D29" s="44" t="inlineStr">
-        <is>
-          <t>仿真草坪</t>
-        </is>
-      </c>
-      <c r="G29" s="45" t="n">
-        <v>30</v>
-      </c>
-      <c r="H29" s="45" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="I29" s="46" t="n">
-        <v>22.450201</v>
-      </c>
-      <c r="K29" s="47" t="inlineStr">
-        <is>
-          <t>中国</t>
-        </is>
-      </c>
-      <c r="M29" s="48" t="inlineStr">
-        <is>
-          <t>美国</t>
-        </is>
-      </c>
-      <c r="P29" s="48" t="inlineStr">
-        <is>
-          <t>义乌(33189)</t>
-        </is>
-      </c>
-      <c r="S29" s="49" t="inlineStr">
-        <is>
-          <t>照章征税</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="D30" s="50" t="inlineStr">
-        <is>
-          <t>0|0|塑料|塑料草坪|无品牌|无型号</t>
-        </is>
-      </c>
-      <c r="G30" s="45" t="n">
-        <v>90</v>
-      </c>
-      <c r="H30" s="45" t="inlineStr">
-        <is>
-          <t>千克</t>
-        </is>
-      </c>
-      <c r="I30" s="46" t="n">
-        <v>673.51</v>
-      </c>
-      <c r="K30" s="47" t="inlineStr">
-        <is>
-          <t>（CHN）</t>
-        </is>
-      </c>
-      <c r="M30" s="47" t="inlineStr">
-        <is>
-          <t>（USA）</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="D31" s="10" t="n"/>
-      <c r="E31" s="10" t="n"/>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="51" t="n">
-        <v>30</v>
-      </c>
-      <c r="H31" s="51" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="I31" s="52" t="inlineStr">
-        <is>
-          <t>美元</t>
-        </is>
-      </c>
-      <c r="J31" s="10" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="B32" s="44" t="n">
-        <v>3918909001</v>
-      </c>
-      <c r="D32" s="44" t="inlineStr">
-        <is>
-          <t>仿真草坪</t>
-        </is>
-      </c>
-      <c r="G32" s="45" t="n">
-        <v>40</v>
-      </c>
-      <c r="H32" s="45" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="I32" s="46" t="n">
-        <v>30.862108</v>
-      </c>
-      <c r="K32" s="47" t="inlineStr">
-        <is>
-          <t>中国</t>
-        </is>
-      </c>
-      <c r="M32" s="48" t="inlineStr">
-        <is>
-          <t>美国</t>
-        </is>
-      </c>
-      <c r="P32" s="48" t="inlineStr">
-        <is>
-          <t>义乌(33189)</t>
-        </is>
-      </c>
-      <c r="S32" s="49" t="inlineStr">
-        <is>
-          <t>照章征税</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="D33" s="50" t="inlineStr">
-        <is>
-          <t>0|0|塑料|塑料草坪|无品牌|无型号</t>
-        </is>
-      </c>
-      <c r="G33" s="45" t="n">
-        <v>168</v>
-      </c>
-      <c r="H33" s="45" t="inlineStr">
-        <is>
-          <t>千克</t>
-        </is>
-      </c>
-      <c r="I33" s="46" t="n">
-        <v>1234.48</v>
-      </c>
-      <c r="K33" s="47" t="inlineStr">
-        <is>
-          <t>（CHN）</t>
-        </is>
-      </c>
-      <c r="M33" s="47" t="inlineStr">
-        <is>
-          <t>（USA）</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="51" t="n">
-        <v>40</v>
-      </c>
-      <c r="H34" s="51" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="I34" s="52" t="inlineStr">
-        <is>
-          <t>美元</t>
-        </is>
-      </c>
-      <c r="J34" s="10" t="n"/>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="82" t="n"/>
+      <c r="L28" s="12" t="n"/>
+      <c r="M28" s="82" t="n"/>
+      <c r="N28" s="12" t="n"/>
+      <c r="O28" s="12" t="n"/>
+      <c r="P28" s="82" t="n"/>
+      <c r="Q28" s="12" t="n"/>
+      <c r="R28" s="12" t="n"/>
+      <c r="S28" s="85" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="128">
+  <mergeCells count="126">
+    <mergeCell ref="P27:R27"/>
     <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K33:L33"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="I26:J26"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="M21:O21"/>
@@ -1706,11 +1920,13 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="P19:R19"/>
     <mergeCell ref="I25:J25"/>
+    <mergeCell ref="P28:R28"/>
     <mergeCell ref="L9:N9"/>
     <mergeCell ref="H3:J3"/>
+    <mergeCell ref="L18:S18"/>
     <mergeCell ref="D21:F22"/>
+    <mergeCell ref="I18:J18"/>
     <mergeCell ref="M24:O24"/>
-    <mergeCell ref="D29:F29"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="A17:K17"/>
@@ -1718,78 +1934,76 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="O11:P11"/>
     <mergeCell ref="I20:J20"/>
-    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="K28:L28"/>
     <mergeCell ref="D24:F25"/>
-    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C3:D3"/>
     <mergeCell ref="M20:O20"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="K30:L30"/>
     <mergeCell ref="G12:H12"/>
+    <mergeCell ref="Q5:S5"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="O10:S10"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="M22:O22"/>
     <mergeCell ref="C15:S15"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="K21:L21"/>
+    <mergeCell ref="M28:O28"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="I32:J32"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="F18:G18"/>
     <mergeCell ref="D27:F28"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="M26:O26"/>
     <mergeCell ref="O4:S4"/>
-    <mergeCell ref="M29:O29"/>
     <mergeCell ref="M23:O23"/>
-    <mergeCell ref="B29:C29"/>
     <mergeCell ref="P9:S9"/>
     <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I33:J33"/>
     <mergeCell ref="K27:L27"/>
     <mergeCell ref="P20:R20"/>
-    <mergeCell ref="P29:R29"/>
     <mergeCell ref="B16:S16"/>
+    <mergeCell ref="J2:N2"/>
     <mergeCell ref="I19:J19"/>
     <mergeCell ref="G8:I8"/>
     <mergeCell ref="K19:L19"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="P21:R21"/>
+    <mergeCell ref="C13:S13"/>
+    <mergeCell ref="K25:L25"/>
     <mergeCell ref="A8:D8"/>
-    <mergeCell ref="D30:F31"/>
+    <mergeCell ref="G2:H2"/>
     <mergeCell ref="G11:H11"/>
-    <mergeCell ref="D32:F32"/>
     <mergeCell ref="P23:R23"/>
+    <mergeCell ref="M25:O25"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="K10:N10"/>
-    <mergeCell ref="M30:O30"/>
-    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="C2:E2"/>
     <mergeCell ref="K6:N6"/>
     <mergeCell ref="D14:S14"/>
-    <mergeCell ref="M33:O33"/>
+    <mergeCell ref="O5:P5"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="I21:J21"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="M32:O32"/>
     <mergeCell ref="M19:O19"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="I23:J23"/>
     <mergeCell ref="K23:L23"/>
     <mergeCell ref="L17:N17"/>
     <mergeCell ref="D20:F20"/>
-    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="Q12:S12"/>
     <mergeCell ref="C7:D7"/>
+    <mergeCell ref="P25:R25"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="K8:N8"/>
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="L3:N3"/>
-    <mergeCell ref="I34:J34"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="R11:S11"/>
     <mergeCell ref="P3:S3"/>
@@ -1798,15 +2012,17 @@
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="K20:L20"/>
     <mergeCell ref="M27:O27"/>
-    <mergeCell ref="P32:R32"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="I22:J22"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="I28:J28"/>
+    <mergeCell ref="K22:L22"/>
     <mergeCell ref="I12:J12"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="A6:D6"/>
+    <mergeCell ref="P24:R24"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="P26:R26"/>
@@ -1814,11 +2030,8 @@
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="O8:S8"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="I29:J29"/>
     <mergeCell ref="O17:S17"/>
-    <mergeCell ref="D33:F34"/>
     <mergeCell ref="P7:S7"/>
-    <mergeCell ref="I31:J31"/>
     <mergeCell ref="G5:J5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>